<commit_message>
Add real 47-prefecture correlation analysis and update figures
- Verified all 47 prefectural minimum wages (2024 & 2025) from MHLW table.
- Verified prefectural non-regular employment rates (2022 Employment Status
  Survey, Table 2-3).
- New cross-prefecture correlation (Pearson r = 0.38, R^2 = 0.15) with
  scatter figure and honest confounding interpretation.
- New essay Section 7; updated abstract, conclusion, and Figure 3 (all 47, 2025).
- Excel workbook gains a 47-prefecture panel with native scatter + trendline.

https://claude.ai/code/session_01Wo91faqRxaMNQidgk2zuDB
</commit_message>
<xml_diff>
--- a/essay_assets/Japan_MinimumWage_Data.xlsx
+++ b/essay_assets/Japan_MinimumWage_Data.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MinWage_NonRegular" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prefectural_2024" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elasticities" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prefecture_Correlation" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +42,9 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -82,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -93,6 +97,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -620,6 +625,132 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Min Wage (2024) vs Non-Regular Share (2022), 47 Prefectures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Prefectures</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <trendline>
+            <trendlineType val="linear"/>
+            <dispRSqr val="1"/>
+            <dispEq val="1"/>
+          </trendline>
+          <xVal>
+            <numRef>
+              <f>'Prefecture_Correlation'!$B$5:$B$51</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Prefecture_Correlation'!$D$5:$D$51</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="1180"/>
+          <min val="940"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Minimum wage 2024 (¥/hour)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="36"/>
+          <min val="26"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Non-regular share 2022 (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -706,6 +837,33 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="6480000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1680,4 +1838,831 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Minimum Wage vs. Non-Regular Employment, All 47 Prefectures</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sources: MHLW FY2025 minimum-wage table (2024 &amp; 2025); 2022 Employment Status Survey, Table 2-3 (non-regular share of all workers).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Prefecture</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Min wage 2024 (¥)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Min wage 2025 (¥)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Non-regular share 2022 (%)</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Pearson r (2024 wage vs non-reg):</t>
+        </is>
+      </c>
+      <c r="I4">
+        <f>CORREL(B5:B51,D5:D51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Hokkaido</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1010</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>1075</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>R-squared:</t>
+        </is>
+      </c>
+      <c r="I5">
+        <f>I4^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Aomori</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>953</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>1029</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>29.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Iwate</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>952</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>29.7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Miyagi</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>973</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>1038</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>30.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Akita</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>951</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>28.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Yamagata</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>955</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>26.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Fukushima</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>955</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>27.8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Ibaraki</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1005</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>1074</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>31.8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Tochigi</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1004</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>1068</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gunma</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>985</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>1063</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>32.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Saitama</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1078</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>1141</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Chiba</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1076</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>1140</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1163</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>1226</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Kanagawa</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>1162</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>1225</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>32.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Niigata</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>985</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>29.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Toyama</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>998</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>1062</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>27.7</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Ishikawa</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>984</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>1054</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>29.2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Fukui</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>984</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>28.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Yamanashi</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>988</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>1052</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Nagano</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>998</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Gifu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1001</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>1065</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>32.7</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Shizuoka</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1034</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>1097</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Aichi</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1077</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>1140</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>32.1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Mie</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1023</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>1087</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>33.4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Shiga</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1017</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>1080</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Kyoto</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1058</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>1122</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>34.2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>1114</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>1177</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>34.1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Hyogo</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1052</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>1116</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>33.9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Nara</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>986</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>1051</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Wakayama</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>980</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>1045</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>30.4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Tottori</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>957</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>1030</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>29.2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Shimane</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>962</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>30.4</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Okayama</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>982</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>1047</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Hiroshima</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1020</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>1085</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>31.2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Yamaguchi</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>979</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>1043</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>30.8</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Tokushima</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>980</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>1046</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>26.6</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Kagawa</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>970</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>1036</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>28.8</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Ehime</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>956</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Kochi</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>952</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>1023</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>28.3</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Fukuoka</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>1057</v>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>34.2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Saga</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>956</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>1030</v>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>30.5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Nagasaki</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>953</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>32.2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Kumamoto</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>952</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>1034</v>
+      </c>
+      <c r="D47" s="5" t="n">
+        <v>29.9</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Oita</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>954</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D48" s="5" t="n">
+        <v>29.6</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Miyazaki</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>952</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>1023</v>
+      </c>
+      <c r="D49" s="5" t="n">
+        <v>30.7</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Kagoshima</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>953</v>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>1026</v>
+      </c>
+      <c r="D50" s="5" t="n">
+        <v>31.6</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Okinawa</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>952</v>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>1023</v>
+      </c>
+      <c r="D51" s="5" t="n">
+        <v>33.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>